<commit_message>
record design decisions, fix 16x vocab to 321128 in xlsx, add oom.md
</commit_message>
<xml_diff>
--- a/examples/mc2/engram_test/engram_test_cases.xlsx
+++ b/examples/mc2/engram_test/engram_test_cases.xlsx
@@ -745,7 +745,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>[[321125, 9216]]</t>
+          <t>[[321128, 9216]]</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>[[321125, 9216]]</t>
+          <t>[[321128, 9216]]</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1559,7 +1559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1629,34 +1629,46 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>divisibility警告</t>
+          <t>shape说明</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>321125 不能被 4 整除: sliced 模式要求 vocab%%world_size==0(numEntriesPerRank 为均匀映射单一属性), perf_sliced__16x_tensor 建议改 [[321128, 9216]]; local 模式不受影响</t>
+          <t>16x 用例 vocab 已定为 321128(可被4整除, numEntriesPerRank=80282); local 与 sliced 同 shape 以维持缓存配对复用</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>OOM提示</t>
+          <t>numTokens&gt;vocab</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>is_graph=1 时 graph 私有池逐档累积: 16x(hidden=9216) 在 token&gt;=8M 时单次输出 72GiB 必然 OOM(91.75GB卡), 详见 oom.md 与设计文档 M5; M5 落地后将按预算自动 SKIP 并汇总</t>
+          <t>允许并保留大档位: 对应 prefill 长上下文/大 batch 真实场景(index 有放回采样, 值域[0,vocab)); 用例将打 WARNING 并标注 repeated-sampling, 不判失败</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>OOM提示</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>is_graph=1 时 graph 私有池逐档累积: 16x(hidden=9216) 在 token&gt;=8M 时单次输出 72GiB 必然 OOM(91.75GB卡), 详见 oom.md 与设计文档 M5; M5 落地后将按预算自动 SKIP 并汇总</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>依赖</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>须先构建安装本仓 torch_extension(分支 engram-fetch-local-mode), 验证: python -c 'from cann_ops_transformer import ElasticBuffer'</t>
         </is>

</xml_diff>